<commit_message>
finished cleaning variable box plus progress on visualisation dashboard
</commit_message>
<xml_diff>
--- a/historical_reference_data/7-10-2025_Pregnancy_Chip_10/cleaned/UNKNOWN071106_014919_0001VRP_PREGNANCY_CHIP_TEST_10_A_CLEANED.xlsx
+++ b/historical_reference_data/7-10-2025_Pregnancy_Chip_10/cleaned/UNKNOWN071106_014919_0001VRP_PREGNANCY_CHIP_TEST_10_A_CLEANED.xlsx
@@ -614,7 +614,11 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Open Purge</t>
+        </is>
+      </c>
       <c r="C2" t="n">
         <v>16</v>
       </c>
@@ -722,7 +726,11 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Start Pump</t>
+        </is>
+      </c>
       <c r="C3" t="n">
         <v>1028</v>
       </c>
@@ -830,7 +838,11 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Purge</t>
+        </is>
+      </c>
       <c r="C4" t="n">
         <v>1038</v>
       </c>
@@ -938,7 +950,11 @@
       <c r="A5" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Purge</t>
+        </is>
+      </c>
       <c r="C5" t="n">
         <v>2038</v>
       </c>
@@ -1046,7 +1062,11 @@
       <c r="A6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Purge</t>
+        </is>
+      </c>
       <c r="C6" t="n">
         <v>3038</v>
       </c>
@@ -1154,7 +1174,11 @@
       <c r="A7" t="n">
         <v>3</v>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Purge</t>
+        </is>
+      </c>
       <c r="C7" t="n">
         <v>4038</v>
       </c>
@@ -1262,7 +1286,11 @@
       <c r="A8" t="n">
         <v>3</v>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Purge</t>
+        </is>
+      </c>
       <c r="C8" t="n">
         <v>5038</v>
       </c>
@@ -1370,7 +1398,11 @@
       <c r="A9" t="n">
         <v>3</v>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Purge</t>
+        </is>
+      </c>
       <c r="C9" t="n">
         <v>6038</v>
       </c>
@@ -1478,7 +1510,11 @@
       <c r="A10" t="n">
         <v>4</v>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Close Purge</t>
+        </is>
+      </c>
       <c r="C10" t="n">
         <v>6048</v>
       </c>
@@ -1586,7 +1622,11 @@
       <c r="A11" t="n">
         <v>5</v>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Change Pump</t>
+        </is>
+      </c>
       <c r="C11" t="n">
         <v>7060</v>
       </c>
@@ -1694,7 +1734,11 @@
       <c r="A12" t="n">
         <v>6</v>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Open Sample</t>
+        </is>
+      </c>
       <c r="C12" t="n">
         <v>7070</v>
       </c>
@@ -1802,7 +1846,11 @@
       <c r="A13" t="n">
         <v>7</v>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C13" t="n">
         <v>8082</v>
       </c>
@@ -1910,7 +1958,11 @@
       <c r="A14" t="n">
         <v>7</v>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C14" t="n">
         <v>8182</v>
       </c>
@@ -2018,7 +2070,11 @@
       <c r="A15" t="n">
         <v>7</v>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C15" t="n">
         <v>8282</v>
       </c>
@@ -2126,7 +2182,11 @@
       <c r="A16" t="n">
         <v>7</v>
       </c>
-      <c r="B16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C16" t="n">
         <v>8382</v>
       </c>
@@ -2234,7 +2294,11 @@
       <c r="A17" t="n">
         <v>7</v>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C17" t="n">
         <v>8482</v>
       </c>
@@ -2342,7 +2406,11 @@
       <c r="A18" t="n">
         <v>7</v>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C18" t="n">
         <v>8582</v>
       </c>
@@ -2450,7 +2518,11 @@
       <c r="A19" t="n">
         <v>7</v>
       </c>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C19" t="n">
         <v>8682</v>
       </c>
@@ -2558,7 +2630,11 @@
       <c r="A20" t="n">
         <v>7</v>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C20" t="n">
         <v>8782</v>
       </c>
@@ -2666,7 +2742,11 @@
       <c r="A21" t="n">
         <v>7</v>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C21" t="n">
         <v>8882</v>
       </c>
@@ -2774,7 +2854,11 @@
       <c r="A22" t="n">
         <v>7</v>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C22" t="n">
         <v>8982</v>
       </c>
@@ -2882,7 +2966,11 @@
       <c r="A23" t="n">
         <v>7</v>
       </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C23" t="n">
         <v>9082</v>
       </c>
@@ -2990,7 +3078,11 @@
       <c r="A24" t="n">
         <v>7</v>
       </c>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C24" t="n">
         <v>9182</v>
       </c>
@@ -3098,7 +3190,11 @@
       <c r="A25" t="n">
         <v>7</v>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C25" t="n">
         <v>9282</v>
       </c>
@@ -3206,7 +3302,11 @@
       <c r="A26" t="n">
         <v>7</v>
       </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C26" t="n">
         <v>9382</v>
       </c>
@@ -3314,7 +3414,11 @@
       <c r="A27" t="n">
         <v>7</v>
       </c>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C27" t="n">
         <v>9482</v>
       </c>
@@ -3422,7 +3526,11 @@
       <c r="A28" t="n">
         <v>7</v>
       </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C28" t="n">
         <v>9582</v>
       </c>
@@ -3530,7 +3638,11 @@
       <c r="A29" t="n">
         <v>7</v>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C29" t="n">
         <v>9682</v>
       </c>
@@ -3638,7 +3750,11 @@
       <c r="A30" t="n">
         <v>7</v>
       </c>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C30" t="n">
         <v>9782</v>
       </c>
@@ -3746,7 +3862,11 @@
       <c r="A31" t="n">
         <v>7</v>
       </c>
-      <c r="B31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C31" t="n">
         <v>9882</v>
       </c>
@@ -3854,7 +3974,11 @@
       <c r="A32" t="n">
         <v>7</v>
       </c>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C32" t="n">
         <v>9982</v>
       </c>
@@ -3962,7 +4086,11 @@
       <c r="A33" t="n">
         <v>7</v>
       </c>
-      <c r="B33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C33" t="n">
         <v>10082</v>
       </c>
@@ -4070,7 +4198,11 @@
       <c r="A34" t="n">
         <v>7</v>
       </c>
-      <c r="B34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C34" t="n">
         <v>10182</v>
       </c>
@@ -4178,7 +4310,11 @@
       <c r="A35" t="n">
         <v>7</v>
       </c>
-      <c r="B35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C35" t="n">
         <v>10282</v>
       </c>
@@ -4286,7 +4422,11 @@
       <c r="A36" t="n">
         <v>7</v>
       </c>
-      <c r="B36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C36" t="n">
         <v>10382</v>
       </c>
@@ -4394,7 +4534,11 @@
       <c r="A37" t="n">
         <v>7</v>
       </c>
-      <c r="B37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C37" t="n">
         <v>10482</v>
       </c>
@@ -4502,7 +4646,11 @@
       <c r="A38" t="n">
         <v>7</v>
       </c>
-      <c r="B38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C38" t="n">
         <v>10582</v>
       </c>
@@ -4610,7 +4758,11 @@
       <c r="A39" t="n">
         <v>7</v>
       </c>
-      <c r="B39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C39" t="n">
         <v>10682</v>
       </c>
@@ -4718,7 +4870,11 @@
       <c r="A40" t="n">
         <v>7</v>
       </c>
-      <c r="B40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C40" t="n">
         <v>10782</v>
       </c>
@@ -4826,7 +4982,11 @@
       <c r="A41" t="n">
         <v>7</v>
       </c>
-      <c r="B41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C41" t="n">
         <v>10882</v>
       </c>
@@ -4934,7 +5094,11 @@
       <c r="A42" t="n">
         <v>7</v>
       </c>
-      <c r="B42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C42" t="n">
         <v>10982</v>
       </c>
@@ -5042,7 +5206,11 @@
       <c r="A43" t="n">
         <v>7</v>
       </c>
-      <c r="B43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C43" t="n">
         <v>11082</v>
       </c>
@@ -5150,7 +5318,11 @@
       <c r="A44" t="n">
         <v>7</v>
       </c>
-      <c r="B44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C44" t="n">
         <v>11182</v>
       </c>
@@ -5258,7 +5430,11 @@
       <c r="A45" t="n">
         <v>7</v>
       </c>
-      <c r="B45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C45" t="n">
         <v>11282</v>
       </c>
@@ -5366,7 +5542,11 @@
       <c r="A46" t="n">
         <v>7</v>
       </c>
-      <c r="B46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C46" t="n">
         <v>11382</v>
       </c>
@@ -5474,7 +5654,11 @@
       <c r="A47" t="n">
         <v>7</v>
       </c>
-      <c r="B47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C47" t="n">
         <v>11482</v>
       </c>
@@ -5582,7 +5766,11 @@
       <c r="A48" t="n">
         <v>7</v>
       </c>
-      <c r="B48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C48" t="n">
         <v>11582</v>
       </c>
@@ -5690,7 +5878,11 @@
       <c r="A49" t="n">
         <v>7</v>
       </c>
-      <c r="B49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C49" t="n">
         <v>11682</v>
       </c>
@@ -5798,7 +5990,11 @@
       <c r="A50" t="n">
         <v>7</v>
       </c>
-      <c r="B50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C50" t="n">
         <v>11782</v>
       </c>
@@ -5906,7 +6102,11 @@
       <c r="A51" t="n">
         <v>7</v>
       </c>
-      <c r="B51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C51" t="n">
         <v>11882</v>
       </c>
@@ -6014,7 +6214,11 @@
       <c r="A52" t="n">
         <v>7</v>
       </c>
-      <c r="B52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C52" t="n">
         <v>11982</v>
       </c>
@@ -6122,7 +6326,11 @@
       <c r="A53" t="n">
         <v>7</v>
       </c>
-      <c r="B53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C53" t="n">
         <v>12082</v>
       </c>
@@ -6230,7 +6438,11 @@
       <c r="A54" t="n">
         <v>7</v>
       </c>
-      <c r="B54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C54" t="n">
         <v>12182</v>
       </c>
@@ -6338,7 +6550,11 @@
       <c r="A55" t="n">
         <v>7</v>
       </c>
-      <c r="B55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C55" t="n">
         <v>12282</v>
       </c>
@@ -6446,7 +6662,11 @@
       <c r="A56" t="n">
         <v>7</v>
       </c>
-      <c r="B56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C56" t="n">
         <v>12382</v>
       </c>
@@ -6554,7 +6774,11 @@
       <c r="A57" t="n">
         <v>7</v>
       </c>
-      <c r="B57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C57" t="n">
         <v>12482</v>
       </c>
@@ -6662,7 +6886,11 @@
       <c r="A58" t="n">
         <v>7</v>
       </c>
-      <c r="B58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C58" t="n">
         <v>12582</v>
       </c>
@@ -6770,7 +6998,11 @@
       <c r="A59" t="n">
         <v>7</v>
       </c>
-      <c r="B59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C59" t="n">
         <v>12682</v>
       </c>
@@ -6878,7 +7110,11 @@
       <c r="A60" t="n">
         <v>7</v>
       </c>
-      <c r="B60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C60" t="n">
         <v>12782</v>
       </c>
@@ -6986,7 +7222,11 @@
       <c r="A61" t="n">
         <v>7</v>
       </c>
-      <c r="B61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C61" t="n">
         <v>12882</v>
       </c>
@@ -7094,7 +7334,11 @@
       <c r="A62" t="n">
         <v>7</v>
       </c>
-      <c r="B62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C62" t="n">
         <v>12982</v>
       </c>
@@ -7202,7 +7446,11 @@
       <c r="A63" t="n">
         <v>7</v>
       </c>
-      <c r="B63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Breath</t>
+        </is>
+      </c>
       <c r="C63" t="n">
         <v>13082</v>
       </c>
@@ -7310,7 +7558,11 @@
       <c r="A64" t="n">
         <v>8</v>
       </c>
-      <c r="B64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Close Sample</t>
+        </is>
+      </c>
       <c r="C64" t="n">
         <v>13092</v>
       </c>
@@ -7418,7 +7670,11 @@
       <c r="A65" t="n">
         <v>9</v>
       </c>
-      <c r="B65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Change Pump</t>
+        </is>
+      </c>
       <c r="C65" t="n">
         <v>14104</v>
       </c>
@@ -7526,7 +7782,11 @@
       <c r="A66" t="n">
         <v>10</v>
       </c>
-      <c r="B66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Open purge</t>
+        </is>
+      </c>
       <c r="C66" t="n">
         <v>14114</v>
       </c>
@@ -7634,7 +7894,11 @@
       <c r="A67" t="n">
         <v>11</v>
       </c>
-      <c r="B67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C67" t="n">
         <v>15126</v>
       </c>
@@ -7742,7 +8006,11 @@
       <c r="A68" t="n">
         <v>11</v>
       </c>
-      <c r="B68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C68" t="n">
         <v>16126</v>
       </c>
@@ -7850,7 +8118,11 @@
       <c r="A69" t="n">
         <v>11</v>
       </c>
-      <c r="B69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C69" t="n">
         <v>17126</v>
       </c>
@@ -7958,7 +8230,11 @@
       <c r="A70" t="n">
         <v>11</v>
       </c>
-      <c r="B70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C70" t="n">
         <v>18126</v>
       </c>
@@ -8066,7 +8342,11 @@
       <c r="A71" t="n">
         <v>11</v>
       </c>
-      <c r="B71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C71" t="n">
         <v>19126</v>
       </c>
@@ -8174,7 +8454,11 @@
       <c r="A72" t="n">
         <v>11</v>
       </c>
-      <c r="B72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C72" t="n">
         <v>20126</v>
       </c>
@@ -8282,7 +8566,11 @@
       <c r="A73" t="n">
         <v>11</v>
       </c>
-      <c r="B73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C73" t="n">
         <v>21126</v>
       </c>
@@ -8390,7 +8678,11 @@
       <c r="A74" t="n">
         <v>11</v>
       </c>
-      <c r="B74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C74" t="n">
         <v>22126</v>
       </c>
@@ -8498,7 +8790,11 @@
       <c r="A75" t="n">
         <v>11</v>
       </c>
-      <c r="B75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C75" t="n">
         <v>23126</v>
       </c>
@@ -8606,7 +8902,11 @@
       <c r="A76" t="n">
         <v>11</v>
       </c>
-      <c r="B76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C76" t="n">
         <v>24126</v>
       </c>
@@ -8714,7 +9014,11 @@
       <c r="A77" t="n">
         <v>11</v>
       </c>
-      <c r="B77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Post purge</t>
+        </is>
+      </c>
       <c r="C77" t="n">
         <v>25126</v>
       </c>
@@ -8822,7 +9126,11 @@
       <c r="A78" t="n">
         <v>12</v>
       </c>
-      <c r="B78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Stop Pump</t>
+        </is>
+      </c>
       <c r="C78" t="n">
         <v>25136</v>
       </c>
@@ -8930,7 +9238,11 @@
       <c r="A79" t="n">
         <v>13</v>
       </c>
-      <c r="B79" t="inlineStr"/>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Close purge</t>
+        </is>
+      </c>
       <c r="C79" t="n">
         <v>25146</v>
       </c>

</xml_diff>